<commit_message>
Implementa upload de dados contábeis com validações e processamento robusto; remove lógica de exclusão anterior e ajusta inserção no banco de dados.
</commit_message>
<xml_diff>
--- a/frontend/xlsx_models/modelo-contabilidade-sejaap.xlsx
+++ b/frontend/xlsx_models/modelo-contabilidade-sejaap.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cirog\OneDrive\Área de Trabalho\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cirog\OneDrive\Área de Trabalho\SejaAP-sistema\frontend\xlsx_models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F99F3BD4-2313-4836-A98F-C6CBB8FADB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE860E6B-64D7-481A-B533-AF12F9B74B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1874E877-0FD3-4790-9ACC-91A92A76085A}"/>
   </bookViews>
@@ -47,7 +47,7 @@
     <t>Valor</t>
   </si>
   <si>
-    <t>Data</t>
+    <t>Data - Registro</t>
   </si>
 </sst>
 </file>
@@ -430,8 +430,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>